<commit_message>
Gases nobles sin atenuación en el FLiBe (AF = 1)
La hoja de cálculo aplicaba AF_FLiBe = 100 también a los gases nobles,
que la sal no retiene (KP-TR-012, Tabla B-4: fracción liberada 1,0), y
subestimaba 100 veces su liberación. Ahora AF_FLiBe = 1 para los gases
nobles y 100 para el resto. Libros *_NUBASE2020.xlsx recalculados,
Anexo C y texto del término fuente actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018SBNNJwQB5jPtNDnHDKz7B
</commit_message>
<xml_diff>
--- a/datos/inventario/Calculosfueradelacontencion_NUBASE2020.xlsx
+++ b/datos/inventario/Calculosfueradelacontencion_NUBASE2020.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="351">
   <si>
     <t xml:space="preserve">Sección transversal efectiva (σ) en barns</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t xml:space="preserve">5.2474 d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AF FLiBe 100/100 → 1 (gas noble, KP-TR-012 Tabla B-4)</t>
   </si>
   <si>
     <t xml:space="preserve">Zr-94</t>
@@ -2572,11 +2575,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="42517636"/>
-        <c:axId val="30550357"/>
+        <c:axId val="79803223"/>
+        <c:axId val="29811935"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="42517636"/>
+        <c:axId val="79803223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2645,7 +2648,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30550357"/>
+        <c:crossAx val="29811935"/>
         <c:crossesAt val="1E-005"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2653,7 +2656,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="30550357"/>
+        <c:axId val="29811935"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -2721,7 +2724,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42517636"/>
+        <c:crossAx val="79803223"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3312,11 +3315,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="5879657"/>
-        <c:axId val="24148077"/>
+        <c:axId val="52389416"/>
+        <c:axId val="95959692"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="5879657"/>
+        <c:axId val="52389416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3385,7 +3388,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24148077"/>
+        <c:crossAx val="95959692"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3393,7 +3396,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24148077"/>
+        <c:axId val="95959692"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -3460,7 +3463,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5879657"/>
+        <c:crossAx val="52389416"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5775,10 +5778,10 @@
         <v>1</v>
       </c>
       <c r="AF18" s="48" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="AG18" s="48" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="AH18" s="38" t="n">
         <v>1</v>
@@ -5788,15 +5791,15 @@
       </c>
       <c r="AJ18" s="49" t="n">
         <f aca="false">$S18*(1/X18)*(1/Z18)*(1/AB18)*(1/AD18)*(1/AF18)*(1/AH18)</f>
-        <v>5556569217.53903</v>
+        <v>555656921753.903</v>
       </c>
       <c r="AK18" s="49" t="n">
         <f aca="false">$S18*(1/Y18)*(1/AA18)*(1/AC18)*(1/AE18)*(1/AG18)*(1/AI18)</f>
-        <v>111131384350.781</v>
+        <v>11113138435078.1</v>
       </c>
       <c r="AL18" s="49" t="n">
         <f aca="false">AK18*0.000000000027</f>
-        <v>3.00054737747107</v>
+        <v>300.054737747107</v>
       </c>
       <c r="AM18" s="49" t="str">
         <f aca="false">B18</f>
@@ -5824,11 +5827,11 @@
       </c>
       <c r="AT18" s="51" t="n">
         <f aca="false">$S18*(1/X18)*(1/Z18)*(1/AB18)*(1/AD18)*(1/AF18)</f>
-        <v>5556569217.53903</v>
+        <v>555656921753.903</v>
       </c>
       <c r="AU18" s="50" t="n">
         <f aca="false">$S18*(1/X18)*(1/Z18)*(1/AB18)*(1/AD18)*(1/AF18)*(1/AH18)</f>
-        <v>5556569217.53903</v>
+        <v>555656921753.903</v>
       </c>
       <c r="AX18" s="50" t="n">
         <f aca="false">AO18</f>
@@ -5852,22 +5855,25 @@
       </c>
       <c r="BC18" s="50" t="n">
         <f aca="false">BB18*(1/AG18)</f>
-        <v>111131384350.781</v>
+        <v>11113138435078.1</v>
       </c>
       <c r="BD18" s="50" t="n">
         <f aca="false">BC18*(1/AI18)</f>
-        <v>111131384350.781</v>
+        <v>11113138435078.1</v>
       </c>
       <c r="BF18" s="36" t="s">
         <v>91</v>
       </c>
       <c r="BG18" s="0" t="n">
         <v>453375.36</v>
+      </c>
+      <c r="BI18" s="36" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C19" s="23" t="n">
         <v>40094</v>
@@ -5948,7 +5954,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C20" s="23" t="n">
         <v>54135</v>
@@ -5960,13 +5966,13 @@
         <v>5.29262E-008</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G20" s="37" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H20" s="41" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I20" s="42"/>
       <c r="J20" s="27"/>
@@ -6041,10 +6047,10 @@
         <v>1</v>
       </c>
       <c r="AF20" s="48" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="AG20" s="48" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="AH20" s="38" t="n">
         <v>1</v>
@@ -6054,15 +6060,15 @@
       </c>
       <c r="AJ20" s="49" t="n">
         <f aca="false">$S20*(1/X20)*(1/Z20)*(1/AB20)*(1/AD20)*(1/AF20)*(1/AH20)</f>
-        <v>779270662.848613</v>
+        <v>77927066284.8613</v>
       </c>
       <c r="AK20" s="49" t="n">
         <f aca="false">$S20*(1/Y20)*(1/AA20)*(1/AC20)*(1/AE20)*(1/AG20)*(1/AI20)</f>
-        <v>15585413256.9723</v>
+        <v>1558541325697.23</v>
       </c>
       <c r="AL20" s="49" t="n">
         <f aca="false">AK20*0.000000000027</f>
-        <v>0.420806157938251</v>
+        <v>42.0806157938251</v>
       </c>
       <c r="AM20" s="49" t="str">
         <f aca="false">B20</f>
@@ -6090,11 +6096,11 @@
       </c>
       <c r="AT20" s="51" t="n">
         <f aca="false">$S20*(1/X20)*(1/Z20)*(1/AB20)*(1/AD20)*(1/AF20)</f>
-        <v>779270662.848613</v>
+        <v>77927066284.8613</v>
       </c>
       <c r="AU20" s="50" t="n">
         <f aca="false">$S20*(1/X20)*(1/Z20)*(1/AB20)*(1/AD20)*(1/AF20)*(1/AH20)</f>
-        <v>779270662.848613</v>
+        <v>77927066284.8613</v>
       </c>
       <c r="AX20" s="50" t="n">
         <f aca="false">AO20</f>
@@ -6118,22 +6124,25 @@
       </c>
       <c r="BC20" s="50" t="n">
         <f aca="false">BB20*(1/AG20)</f>
-        <v>15585413256.9723</v>
+        <v>1558541325697.23</v>
       </c>
       <c r="BD20" s="50" t="n">
         <f aca="false">BC20*(1/AI20)</f>
-        <v>15585413256.9723</v>
+        <v>1558541325697.23</v>
       </c>
       <c r="BF20" s="36" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="BG20" s="0" t="n">
         <v>32904</v>
+      </c>
+      <c r="BI20" s="36" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="22" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C21" s="23" t="n">
         <v>40096</v>
@@ -6209,30 +6218,30 @@
       <c r="AL21" s="35"/>
       <c r="AM21" s="35"/>
       <c r="BF21" s="36" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>53129</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E22" s="37" t="n">
         <v>1.74196E-005</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H22" s="41" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I22" s="42" t="n">
         <v>15700000</v>
@@ -6393,7 +6402,7 @@
         <v>165.693802599008</v>
       </c>
       <c r="BF22" s="36" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BG22" s="0" t="n">
         <v>509328786931200</v>
@@ -6401,7 +6410,7 @@
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" s="23" t="n">
         <v>42095</v>
@@ -6482,7 +6491,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C24" s="23" t="n">
         <v>42097</v>
@@ -6563,7 +6572,7 @@
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" s="23" t="n">
         <v>42098</v>
@@ -6644,7 +6653,7 @@
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C26" s="23" t="n">
         <v>42100</v>
@@ -6720,30 +6729,30 @@
       <c r="AL26" s="35"/>
       <c r="AM26" s="35"/>
       <c r="BF26" s="36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C27" s="23" t="n">
         <v>43099</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E27" s="37" t="n">
         <v>0.000135738</v>
       </c>
       <c r="F27" s="37" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G27" s="37" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H27" s="41" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I27" s="42" t="n">
         <v>213000</v>
@@ -6904,7 +6913,7 @@
         <v>3290.51272728106</v>
       </c>
       <c r="BF27" s="36" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="BG27" s="0" t="n">
         <v>6661667095488</v>
@@ -6912,7 +6921,7 @@
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C28" s="23" t="n">
         <v>44100</v>
@@ -6993,7 +7002,7 @@
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C29" s="23" t="n">
         <v>44101</v>
@@ -7074,7 +7083,7 @@
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C30" s="23" t="n">
         <v>44102</v>
@@ -7155,25 +7164,25 @@
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C31" s="23" t="n">
         <v>44103</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E31" s="37" t="n">
         <v>2.04804E-005</v>
       </c>
       <c r="F31" s="37" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G31" s="37" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H31" s="41" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I31" s="42"/>
       <c r="J31" s="27" t="n">
@@ -7334,7 +7343,7 @@
         <v>975405979.291832</v>
       </c>
       <c r="BF31" s="36" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="BG31" s="0" t="n">
         <v>3390768</v>
@@ -7342,7 +7351,7 @@
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C32" s="23" t="n">
         <v>44104</v>
@@ -7423,25 +7432,25 @@
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C33" s="23" t="n">
         <v>44106</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E33" s="37" t="n">
         <v>2.6273E-005</v>
       </c>
       <c r="F33" s="37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G33" s="37" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H33" s="41" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I33" s="42"/>
       <c r="J33" s="27" t="n">
@@ -7602,7 +7611,7 @@
         <v>132078337.213248</v>
       </c>
       <c r="BF33" s="36" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="BG33" s="0" t="n">
         <v>32123520</v>
@@ -7610,7 +7619,7 @@
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C34" s="23" t="n">
         <v>45103</v>
@@ -7691,23 +7700,23 @@
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" s="23" t="n">
         <v>45105</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E35" s="37" t="n">
         <v>4.30968E-007</v>
       </c>
       <c r="F35" s="37"/>
       <c r="G35" s="37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H35" s="41" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I35" s="42"/>
       <c r="J35" s="27"/>
@@ -7868,7 +7877,7 @@
         <v>547026977.069659</v>
       </c>
       <c r="BF35" s="36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="BG35" s="0" t="n">
         <v>127227.6</v>
@@ -7876,7 +7885,7 @@
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C36" s="23" t="n">
         <v>46105</v>
@@ -7957,7 +7966,7 @@
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C37" s="23" t="n">
         <v>46106</v>
@@ -8038,25 +8047,25 @@
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C38" s="23" t="n">
         <v>92235</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E38" s="37" t="n">
         <v>0.00223551</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H38" s="41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I38" s="59" t="n">
         <v>703800000</v>
@@ -8217,7 +8226,7 @@
         <v>0.812501786310237</v>
       </c>
       <c r="BF38" s="36" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="BG38" s="0" t="n">
         <v>22216075960320000</v>
@@ -8225,7 +8234,7 @@
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C39" s="23" t="n">
         <v>46108</v>
@@ -8306,7 +8315,7 @@
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C40" s="23" t="n">
         <v>47109</v>
@@ -8387,7 +8396,7 @@
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C41" s="23" t="n">
         <v>52130</v>
@@ -8463,30 +8472,30 @@
       <c r="AL41" s="35"/>
       <c r="AM41" s="35"/>
       <c r="BF41" s="36" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="22" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C42" s="23" t="n">
         <v>92237</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E42" s="37" t="n">
         <v>2.84647E-006</v>
       </c>
       <c r="F42" s="37" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G42" s="37" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H42" s="41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I42" s="63"/>
       <c r="J42" s="64"/>
@@ -8647,7 +8656,7 @@
         <v>39398119.5869155</v>
       </c>
       <c r="BF42" s="36" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="BG42" s="0" t="n">
         <v>583372.8</v>
@@ -8655,7 +8664,7 @@
     </row>
     <row r="43" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C43" s="23" t="n">
         <v>54131</v>
@@ -8736,7 +8745,7 @@
     </row>
     <row r="44" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C44" s="23" t="n">
         <v>54132</v>
@@ -8817,25 +8826,25 @@
     </row>
     <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C45" s="23" t="n">
         <v>92238</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E45" s="37" t="n">
         <v>0.0179355</v>
       </c>
       <c r="F45" s="37" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G45" s="37" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H45" s="41" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I45" s="59" t="n">
         <v>4468000000</v>
@@ -8996,7 +9005,7 @@
         <v>1.02826953307641</v>
       </c>
       <c r="BF45" s="36" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="BG45" s="0" t="n">
         <v>1.4083856109504E+017</v>
@@ -9004,7 +9013,7 @@
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C46" s="23" t="n">
         <v>54134</v>
@@ -9085,25 +9094,25 @@
     </row>
     <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C47" s="23" t="n">
         <v>93237</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E47" s="37" t="n">
         <v>3.07925E-005</v>
       </c>
       <c r="F47" s="37" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G47" s="37" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H47" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I47" s="59"/>
       <c r="J47" s="27" t="n">
@@ -9264,7 +9273,7 @@
         <v>3.67485777634551</v>
       </c>
       <c r="BF47" s="36" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="BG47" s="0" t="n">
         <v>67658049515520</v>
@@ -9272,7 +9281,7 @@
     </row>
     <row r="48" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C48" s="23" t="n">
         <v>54136</v>
@@ -9348,12 +9357,12 @@
       <c r="AL48" s="35"/>
       <c r="AM48" s="35"/>
       <c r="BF48" s="36" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C49" s="23" t="n">
         <v>55133</v>
@@ -9434,7 +9443,7 @@
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C50" s="23" t="n">
         <v>55134</v>
@@ -9446,13 +9455,13 @@
         <v>1.72686E-005</v>
       </c>
       <c r="F50" s="37" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G50" s="37" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H50" s="22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I50" s="26"/>
       <c r="J50" s="27"/>
@@ -9605,36 +9614,36 @@
         <v>2139722436.40049</v>
       </c>
       <c r="BF50" s="36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="BG50" s="0" t="n">
         <v>65165052.3552</v>
       </c>
       <c r="BI50" s="36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C51" s="23" t="n">
         <v>93239</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E51" s="37" t="n">
         <v>1.71895E-005</v>
       </c>
       <c r="F51" s="37" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G51" s="37" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H51" s="41" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I51" s="59"/>
       <c r="J51" s="27"/>
@@ -9795,7 +9804,7 @@
         <v>681850675.2662</v>
       </c>
       <c r="BF51" s="36" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="BG51" s="0" t="n">
         <v>203558.4</v>
@@ -9803,25 +9812,25 @@
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C52" s="23" t="n">
         <v>94238</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E52" s="37" t="n">
         <v>8.29987E-006</v>
       </c>
       <c r="F52" s="37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G52" s="37" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H52" s="41" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I52" s="59" t="n">
         <v>87.7</v>
@@ -9982,7 +9991,7 @@
         <v>24215.4232033186</v>
       </c>
       <c r="BF52" s="36" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="BG52" s="0" t="n">
         <v>2767542417.216</v>
@@ -9990,25 +9999,25 @@
     </row>
     <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="22" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C53" s="23" t="n">
         <v>94239</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E53" s="37" t="n">
         <v>0.000258547</v>
       </c>
       <c r="F53" s="37" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G53" s="37" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H53" s="41" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I53" s="59" t="n">
         <v>24100</v>
@@ -10169,7 +10178,7 @@
         <v>2743.86448959861</v>
       </c>
       <c r="BF53" s="36" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="BG53" s="0" t="n">
         <v>760837487788.8</v>
@@ -10177,25 +10186,25 @@
     </row>
     <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="22" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C54" s="23" t="n">
         <v>94240</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E54" s="37" t="n">
         <v>7.855E-005</v>
       </c>
       <c r="F54" s="37" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G54" s="37" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H54" s="41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I54" s="59" t="n">
         <v>6560</v>
@@ -10356,7 +10365,7 @@
         <v>3063.34928603926</v>
       </c>
       <c r="BF54" s="36" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="BG54" s="0" t="n">
         <v>207044992010.88</v>
@@ -10364,7 +10373,7 @@
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C55" s="23" t="n">
         <v>57139</v>
@@ -10445,25 +10454,25 @@
     </row>
     <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="22" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C56" s="23" t="n">
         <v>94241</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E56" s="37" t="n">
         <v>7.80575E-005</v>
       </c>
       <c r="F56" s="37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G56" s="37" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H56" s="41" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I56" s="59" t="n">
         <v>14.3</v>
@@ -10624,7 +10633,7 @@
         <v>1393859.89261286</v>
       </c>
       <c r="BF56" s="36" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="BG56" s="0" t="n">
         <v>452179193.80032</v>
@@ -10632,25 +10641,25 @@
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C57" s="23" t="n">
         <v>94242</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E57" s="37" t="n">
         <v>2.86215E-005</v>
       </c>
       <c r="F57" s="37" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G57" s="37" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H57" s="41" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I57" s="59" t="n">
         <v>375000</v>
@@ -10811,7 +10820,7 @@
         <v>19.5290667374305</v>
       </c>
       <c r="BF57" s="36" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="BG57" s="0" t="n">
         <v>11833847280000</v>
@@ -10819,25 +10828,25 @@
     </row>
     <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C58" s="23" t="n">
         <v>95241</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E58" s="37" t="n">
         <v>6.97773E-007</v>
       </c>
       <c r="F58" s="37" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G58" s="37" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H58" s="41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I58" s="59" t="n">
         <v>14.4</v>
@@ -10998,7 +11007,7 @@
         <v>412.712870105851</v>
       </c>
       <c r="BF58" s="36" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="BG58" s="0" t="n">
         <v>13651526222.208</v>
@@ -11006,25 +11015,25 @@
     </row>
     <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C59" s="23" t="n">
         <v>95243</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E59" s="37" t="n">
         <v>5.53963E-006</v>
       </c>
       <c r="F59" s="37" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G59" s="37" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H59" s="41" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I59" s="59"/>
       <c r="J59" s="27"/>
@@ -11185,7 +11194,7 @@
         <v>192.847399166304</v>
       </c>
       <c r="BF59" s="36" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="BG59" s="0" t="n">
         <v>231943406688</v>
@@ -11193,25 +11202,25 @@
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="22" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C60" s="23" t="n">
         <v>38089</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E60" s="37" t="n">
         <v>2.33352E-005</v>
       </c>
       <c r="F60" s="37" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G60" s="37" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H60" s="22" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I60" s="26"/>
       <c r="J60" s="67" t="n">
@@ -11372,7 +11381,7 @@
         <v>43130054867.596</v>
       </c>
       <c r="BF60" s="36" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="BG60" s="0" t="n">
         <v>4368643.2</v>
@@ -11380,25 +11389,25 @@
     </row>
     <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B61" s="22" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C61" s="23" t="n">
         <v>38090</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E61" s="37" t="n">
         <v>0.000123058</v>
       </c>
       <c r="F61" s="37" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G61" s="37" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H61" s="22" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I61" s="26" t="n">
         <v>28.8</v>
@@ -11559,7 +11568,7 @@
         <v>1089136035.42421</v>
       </c>
       <c r="BF61" s="36" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="BG61" s="0" t="n">
         <v>912310732.9728</v>
@@ -11567,13 +11576,13 @@
     </row>
     <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B62" s="22" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C62" s="23" t="n">
         <v>56138</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E62" s="37" t="n">
         <v>0.000167617</v>
@@ -11583,7 +11592,7 @@
         <v>53</v>
       </c>
       <c r="H62" s="41" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I62" s="42" t="n">
         <f aca="false">30.018</f>
@@ -11750,25 +11759,25 @@
     </row>
     <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B63" s="22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C63" s="23" t="n">
         <v>56140</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E63" s="37" t="n">
         <v>1.10185E-005</v>
       </c>
       <c r="F63" s="37" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G63" s="37" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H63" s="41" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="I63" s="42"/>
       <c r="J63" s="27" t="n">
@@ -11929,7 +11938,7 @@
         <v>80741685570.4183</v>
       </c>
       <c r="BF63" s="36" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="BG63" s="0" t="n">
         <v>1101893.76</v>
@@ -11937,23 +11946,23 @@
     </row>
     <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B64" s="22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C64" s="23" t="n">
         <v>61147</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E64" s="37" t="n">
         <v>2.53495E-005</v>
       </c>
       <c r="F64" s="37"/>
       <c r="G64" s="37" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H64" s="41" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I64" s="59"/>
       <c r="J64" s="27"/>
@@ -12112,37 +12121,37 @@
         <v>4944874.1812184</v>
       </c>
       <c r="BF64" s="36" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="BG64" s="0" t="n">
         <v>82786439.878272</v>
       </c>
       <c r="BH64" s="36" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="BI64" s="36" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="69" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C65" s="70" t="n">
         <v>61149</v>
       </c>
       <c r="D65" s="70" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E65" s="71" t="n">
         <v>3.50308E-007</v>
       </c>
       <c r="F65" s="71"/>
       <c r="G65" s="71" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H65" s="72" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I65" s="73"/>
       <c r="J65" s="61"/>
@@ -12301,39 +12310,39 @@
         <v>29604770.2699976</v>
       </c>
       <c r="BF65" s="36" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="BG65" s="0" t="n">
         <v>191088</v>
       </c>
       <c r="BH65" s="36" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="BI65" s="36" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B66" s="22" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C66" s="23" t="n">
         <v>39091</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E66" s="37" t="n">
         <v>3.29343E-005</v>
       </c>
       <c r="F66" s="37" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G66" s="37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H66" s="22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="I66" s="80"/>
       <c r="J66" s="28" t="n">
@@ -12492,7 +12501,7 @@
         <v>1052082148.08156</v>
       </c>
       <c r="BF66" s="36" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="BG66" s="0" t="n">
         <v>5055264</v>
@@ -12500,7 +12509,7 @@
     </row>
     <row r="67" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B67" s="81" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C67" s="82" t="n">
         <v>60148</v>
@@ -12585,25 +12594,25 @@
     </row>
     <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="22" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C68" s="23" t="n">
         <v>40093</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E68" s="37" t="n">
         <v>0.000143526</v>
       </c>
       <c r="F68" s="37" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G68" s="37" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H68" s="41" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I68" s="42" t="n">
         <v>1530000</v>
@@ -12762,7 +12771,7 @@
         <v>456.199776070118</v>
       </c>
       <c r="BF68" s="36" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="BG68" s="0" t="n">
         <v>50806650988800</v>
@@ -12770,25 +12779,25 @@
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B69" s="22" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C69" s="23" t="n">
         <v>40095</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E69" s="37" t="n">
         <v>4.35054E-005</v>
       </c>
       <c r="F69" s="37" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G69" s="37" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H69" s="41" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I69" s="42"/>
       <c r="J69" s="27" t="n">
@@ -12947,7 +12956,7 @@
         <v>1269923065.93952</v>
       </c>
       <c r="BF69" s="36" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="BG69" s="0" t="n">
         <v>5532364.8</v>
@@ -12955,25 +12964,25 @@
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B70" s="22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C70" s="23" t="n">
         <v>41095</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E70" s="37" t="n">
         <v>2.02169E-005</v>
       </c>
       <c r="F70" s="37" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G70" s="37" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H70" s="22" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="I70" s="26"/>
       <c r="J70" s="27" t="n">
@@ -13132,7 +13141,7 @@
         <v>1079914869.44097</v>
       </c>
       <c r="BF70" s="36" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="BG70" s="0" t="n">
         <v>3023222.4</v>
@@ -13140,23 +13149,23 @@
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B71" s="88" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C71" s="23" t="n">
         <v>58140</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E71" s="37" t="n">
         <v>0.000141465</v>
       </c>
       <c r="F71" s="37"/>
       <c r="G71" s="37" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H71" s="41" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I71" s="59"/>
       <c r="J71" s="27"/>
@@ -13318,28 +13327,28 @@
         <v>54</v>
       </c>
       <c r="BH71" s="36" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B72" s="88" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C72" s="23" t="n">
         <v>58141</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E72" s="37" t="n">
         <v>2.33596E-005</v>
       </c>
       <c r="F72" s="37"/>
       <c r="G72" s="37" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H72" s="41" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I72" s="59"/>
       <c r="J72" s="27"/>
@@ -13498,24 +13507,24 @@
         <v>134321812.63423</v>
       </c>
       <c r="BF72" s="36" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="BG72" s="0" t="n">
         <v>2808432</v>
       </c>
       <c r="BH72" s="36" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B73" s="88" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C73" s="23" t="n">
         <v>58142</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E73" s="37" t="n">
         <v>0.000144249</v>
@@ -13525,7 +13534,7 @@
         <v>53</v>
       </c>
       <c r="H73" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I73" s="59"/>
       <c r="J73" s="27"/>
@@ -13687,28 +13696,28 @@
         <v>54</v>
       </c>
       <c r="BH73" s="36" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B74" s="88" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C74" s="23" t="n">
         <v>58144</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E74" s="37" t="n">
         <v>8.66279E-005</v>
       </c>
       <c r="F74" s="37"/>
       <c r="G74" s="37" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H74" s="41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="I74" s="59"/>
       <c r="J74" s="27"/>
@@ -13867,34 +13876,34 @@
         <v>56835278.3728631</v>
       </c>
       <c r="BF74" s="36" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="BG74" s="0" t="n">
         <v>24614150.4</v>
       </c>
       <c r="BH74" s="36" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B75" s="88" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C75" s="23" t="n">
         <v>59141</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E75" s="37" t="n">
         <v>0.000116698</v>
       </c>
       <c r="F75" s="37"/>
       <c r="G75" s="37" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H75" s="41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="I75" s="59"/>
       <c r="J75" s="27"/>
@@ -14056,28 +14065,28 @@
         <v>54</v>
       </c>
       <c r="BH75" s="36" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="88" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C76" s="23" t="n">
         <v>59143</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E76" s="37" t="n">
         <v>1.0667E-005</v>
       </c>
       <c r="F76" s="37"/>
       <c r="G76" s="37" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H76" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I76" s="59"/>
       <c r="J76" s="27"/>
@@ -14236,24 +14245,24 @@
         <v>146924343.834602</v>
       </c>
       <c r="BF76" s="36" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="BG76" s="0" t="n">
         <v>1172448</v>
       </c>
       <c r="BH76" s="36" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B77" s="88" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C77" s="23" t="n">
         <v>60143</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E77" s="37" t="n">
         <v>0.000100964</v>
@@ -14263,7 +14272,7 @@
         <v>53</v>
       </c>
       <c r="H77" s="41" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I77" s="59"/>
       <c r="J77" s="27"/>
@@ -14427,23 +14436,23 @@
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B78" s="88" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C78" s="23" t="n">
         <v>60144</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E78" s="37" t="n">
         <v>7.13987E-005</v>
       </c>
       <c r="F78" s="37"/>
       <c r="G78" s="37" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H78" s="41" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I78" s="59"/>
       <c r="J78" s="27"/>
@@ -14602,12 +14611,12 @@
         <v>0</v>
       </c>
       <c r="BF78" s="36" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B79" s="22" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C79" s="23" t="n">
         <v>64157</v>
@@ -14692,13 +14701,13 @@
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B80" s="88" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C80" s="23" t="n">
         <v>60145</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E80" s="37" t="n">
         <v>8.47874E-005</v>
@@ -14708,7 +14717,7 @@
         <v>53</v>
       </c>
       <c r="H80" s="41" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="I80" s="59"/>
       <c r="J80" s="27"/>
@@ -14872,25 +14881,25 @@
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B81" s="22" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C81" s="23" t="n">
         <v>92236</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E81" s="37" t="n">
         <v>0.000433584</v>
       </c>
       <c r="F81" s="37" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G81" s="37" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="H81" s="41" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I81" s="59"/>
       <c r="J81" s="27"/>
@@ -15043,24 +15052,24 @@
         <v>4.73703641791764</v>
       </c>
       <c r="BF81" s="36" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="BG81" s="0" t="n">
         <v>739063208793600</v>
       </c>
       <c r="BI81" s="36" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B82" s="88" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C82" s="23" t="n">
         <v>60146</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E82" s="37" t="n">
         <v>8.23345E-005</v>
@@ -15070,7 +15079,7 @@
         <v>53</v>
       </c>
       <c r="H82" s="41" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="I82" s="59"/>
       <c r="J82" s="27" t="n">
@@ -15234,25 +15243,25 @@
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B83" s="88" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C83" s="23" t="n">
         <v>60147</v>
       </c>
       <c r="D83" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E83" s="37" t="n">
         <v>3.36571E-006</v>
       </c>
       <c r="F83" s="37" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G83" s="37" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H83" s="41" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I83" s="59"/>
       <c r="J83" s="27"/>
@@ -15411,7 +15420,7 @@
         <v>57293541.1232211</v>
       </c>
       <c r="BF83" s="36" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="BG83" s="0" t="n">
         <v>948672</v>
@@ -15419,13 +15428,13 @@
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B84" s="88" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C84" s="23" t="n">
         <v>60150</v>
       </c>
       <c r="D84" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E84" s="37" t="n">
         <v>1.83824E-005</v>
@@ -15435,7 +15444,7 @@
         <v>53</v>
       </c>
       <c r="H84" s="41" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="I84" s="59" t="n">
         <v>7E+018</v>
@@ -15594,30 +15603,30 @@
         <v>0</v>
       </c>
       <c r="BF84" s="36" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B85" s="88" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C85" s="23" t="n">
         <v>62147</v>
       </c>
       <c r="D85" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E85" s="37" t="n">
         <v>3.14028E-006</v>
       </c>
       <c r="F85" s="37" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G85" s="37" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="H85" s="41" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I85" s="59"/>
       <c r="J85" s="27"/>
@@ -15776,34 +15785,34 @@
         <v>1.50751461391606E-005</v>
       </c>
       <c r="BF85" s="36" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="BG85" s="0" t="n">
         <v>3.363968320128E+018</v>
       </c>
       <c r="BH85" s="36" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B86" s="88" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C86" s="23" t="n">
         <v>62149</v>
       </c>
       <c r="D86" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E86" s="37" t="n">
         <v>3.24339E-007</v>
       </c>
       <c r="F86" s="37"/>
       <c r="G86" s="37" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H86" s="41" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I86" s="59"/>
       <c r="J86" s="27"/>
@@ -15965,18 +15974,18 @@
         <v>54</v>
       </c>
       <c r="BH86" s="36" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B87" s="88" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C87" s="23" t="n">
         <v>62150</v>
       </c>
       <c r="D87" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E87" s="37" t="n">
         <v>2.42831E-005</v>
@@ -15986,7 +15995,7 @@
         <v>53</v>
       </c>
       <c r="H87" s="41" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I87" s="59"/>
       <c r="J87" s="27"/>
@@ -16148,28 +16157,28 @@
         <v>54</v>
       </c>
       <c r="BH87" s="36" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B88" s="88" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C88" s="23" t="n">
         <v>62151</v>
       </c>
       <c r="D88" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E88" s="37" t="n">
         <v>1.86627E-006</v>
       </c>
       <c r="F88" s="37"/>
       <c r="G88" s="37" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="H88" s="41" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I88" s="59"/>
       <c r="J88" s="27"/>
@@ -16328,24 +16337,24 @@
         <v>10095.6364006612</v>
       </c>
       <c r="BF88" s="36" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="BG88" s="0" t="n">
         <v>2985285207.168</v>
       </c>
       <c r="BH88" s="36" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B89" s="88" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C89" s="23" t="n">
         <v>62152</v>
       </c>
       <c r="D89" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E89" s="37" t="n">
         <v>1.06573E-005</v>
@@ -16355,7 +16364,7 @@
         <v>53</v>
       </c>
       <c r="H89" s="41" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="I89" s="59"/>
       <c r="J89" s="27"/>
@@ -16517,28 +16526,28 @@
         <v>54</v>
       </c>
       <c r="BH89" s="36" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B90" s="88" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C90" s="23" t="n">
         <v>63153</v>
       </c>
       <c r="D90" s="23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E90" s="37" t="n">
         <v>1.08169E-005</v>
       </c>
       <c r="F90" s="37"/>
       <c r="G90" s="37" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="H90" s="41" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="I90" s="59"/>
       <c r="J90" s="27"/>
@@ -16700,28 +16709,28 @@
         <v>54</v>
       </c>
       <c r="BH90" s="36" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B91" s="88" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C91" s="23" t="n">
         <v>63154</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E91" s="37" t="n">
         <v>1.93525E-006</v>
       </c>
       <c r="F91" s="37"/>
       <c r="G91" s="37" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="H91" s="41" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="I91" s="59"/>
       <c r="J91" s="27"/>
@@ -16882,37 +16891,37 @@
         <v>57631931.4353424</v>
       </c>
       <c r="BF91" s="36" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="BG91" s="0" t="n">
         <v>271137108.87936</v>
       </c>
       <c r="BH91" s="36" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="BI91" s="36" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B92" s="88" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C92" s="23" t="n">
         <v>63155</v>
       </c>
       <c r="D92" s="23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E92" s="37" t="n">
         <v>5.7612E-007</v>
       </c>
       <c r="F92" s="37"/>
       <c r="G92" s="37" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H92" s="41" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I92" s="59"/>
       <c r="J92" s="27"/>
@@ -17073,16 +17082,16 @@
         <v>31086495.7822499</v>
       </c>
       <c r="BF92" s="36" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="BG92" s="0" t="n">
         <v>149642943.47136</v>
       </c>
       <c r="BH92" s="36" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="BI92" s="36" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -17090,10 +17099,10 @@
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G96" s="0" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J96" s="89" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17101,7 +17110,7 @@
         <v>87</v>
       </c>
       <c r="J97" s="89" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="K97" s="89" t="n">
         <v>120</v>
@@ -17109,10 +17118,10 @@
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G98" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J98" s="89" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="K98" s="89" t="n">
         <v>309</v>
@@ -17125,7 +17134,7 @@
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G100" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17135,22 +17144,22 @@
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G102" s="0" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G103" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G104" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="G105" s="0" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18461,7 +18470,7 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D7" s="49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E7" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX51</f>
@@ -18518,16 +18527,16 @@
       </c>
       <c r="J8" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!BC18</f>
-        <v>111131384350.781</v>
+        <v>11113138435078.1</v>
       </c>
       <c r="K8" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!BD18</f>
-        <v>111131384350.781</v>
+        <v>11113138435078.1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="49" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E9" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX63</f>
@@ -18560,7 +18569,7 @@
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D10" s="49" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E10" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX76</f>
@@ -18593,7 +18602,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D11" s="49" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E11" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX72</f>
@@ -18626,7 +18635,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D12" s="49" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E12" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX69</f>
@@ -18659,7 +18668,7 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="49" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E13" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX70</f>
@@ -18692,7 +18701,7 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="49" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E14" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX66</f>
@@ -18725,7 +18734,7 @@
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D15" s="49" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E15" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX31</f>
@@ -18758,7 +18767,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D16" s="49" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E16" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX60</f>
@@ -18791,7 +18800,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D17" s="49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E17" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX42</f>
@@ -18824,7 +18833,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D18" s="49" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E18" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX83</f>
@@ -18857,7 +18866,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D19" s="49" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E19" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX74</f>
@@ -18890,7 +18899,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D20" s="49" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E20" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX35</f>
@@ -18923,7 +18932,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D21" s="49" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E21" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX65</f>
@@ -18956,7 +18965,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D22" s="49" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E22" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX20</f>
@@ -18980,16 +18989,16 @@
       </c>
       <c r="J22" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!BC20</f>
-        <v>15585413256.9723</v>
+        <v>1558541325697.23</v>
       </c>
       <c r="K22" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!BD20</f>
-        <v>15585413256.9723</v>
+        <v>1558541325697.23</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D23" s="49" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E23" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX33</f>
@@ -19022,7 +19031,7 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D24" s="49" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E24" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX64</f>
@@ -19055,7 +19064,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D25" s="49" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E25" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX50</f>
@@ -19088,7 +19097,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D26" s="49" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E26" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX56</f>
@@ -19154,7 +19163,7 @@
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D28" s="49" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E28" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX61</f>
@@ -19187,7 +19196,7 @@
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D29" s="49" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E29" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX91</f>
@@ -19220,7 +19229,7 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D30" s="49" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E30" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX92</f>
@@ -19253,7 +19262,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D31" s="49" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E31" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX52</f>
@@ -19286,7 +19295,7 @@
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D32" s="49" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E32" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX88</f>
@@ -19319,7 +19328,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D33" s="49" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E33" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX54</f>
@@ -19352,7 +19361,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D34" s="49" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E34" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX53</f>
@@ -19385,7 +19394,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D35" s="79" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E35" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX58</f>
@@ -19418,7 +19427,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D36" s="49" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E36" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX59</f>
@@ -19451,7 +19460,7 @@
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D37" s="49" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E37" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX27</f>
@@ -19484,7 +19493,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D38" s="49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E38" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX68</f>
@@ -19517,7 +19526,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D39" s="49" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E39" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX57</f>
@@ -19583,7 +19592,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D41" s="49" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E41" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX81</f>
@@ -19616,7 +19625,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D42" s="49" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E42" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX47</f>
@@ -19649,7 +19658,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D43" s="49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E43" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX45</f>
@@ -19715,7 +19724,7 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D45" s="49" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E45" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX38</f>
@@ -19748,7 +19757,7 @@
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D46" s="49" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E46" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX22</f>
@@ -19814,7 +19823,7 @@
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D48" s="49" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E48" s="50" t="n">
         <f aca="false">'AZ6 RZ1 (ACCIDENT)'!AX85</f>
@@ -19857,7 +19866,7 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D50" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E50" s="50"/>
       <c r="F50" s="50"/>

</xml_diff>